<commit_message>
Fix person import sample columns
</commit_message>
<xml_diff>
--- a/sample-data/Mau_Import_NhanKhau.xlsx
+++ b/sample-data/Mau_Import_NhanKhau.xlsx
@@ -497,13 +497,13 @@
         <v>Chủ hộ</v>
       </c>
       <c r="K2" s="6" t="str">
-        <v>Nông nghiệp</v>
+        <v>Kinh</v>
       </c>
       <c r="L2" s="6" t="str">
-        <v>Kinh</v>
+        <v>Không</v>
       </c>
       <c r="M2" s="6" t="str">
-        <v>Không</v>
+        <v>Nông nghiệp</v>
       </c>
       <c r="N2" s="6" t="str">
         <v>12/12</v>

</xml_diff>